<commit_message>
chore(templates): internal tester row on all Collection Schedule workbooks
Adds add_internal_tester_row.py: row 2 Stand {{########}}, Alex Nyandoro, deposit 5000, total 120000, +17785808657, alex@michaeltenable.com, Internal Tester; J=N; K=(I-H)/N; start 5 May 2026. Updates all 9 xlsx templates and README.

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/docs/payment-schedule-templates/Payment Schedules - Customer Portal/Collection_Schedule_Template_120mo.xlsx
+++ b/docs/payment-schedule-templates/Payment Schedules - Customer Portal/Collection_Schedule_Template_120mo.xlsx
@@ -1487,20 +1487,55 @@
       </c>
     </row>
     <row r="2" ht="15" customHeight="1" s="14">
-      <c r="A2" s="20" t="n"/>
-      <c r="B2" s="20" t="n"/>
-      <c r="C2" s="20" t="n"/>
-      <c r="D2" s="20" t="n"/>
-      <c r="E2" s="20" t="n"/>
-      <c r="F2" s="20" t="n"/>
-      <c r="G2" s="21" t="n"/>
-      <c r="H2" s="21" t="n"/>
-      <c r="I2" s="21" t="n"/>
+      <c r="A2" s="20" t="inlineStr">
+        <is>
+          <t>{{########}}</t>
+        </is>
+      </c>
+      <c r="B2" s="20" t="inlineStr">
+        <is>
+          <t>Alex</t>
+        </is>
+      </c>
+      <c r="C2" s="20" t="inlineStr">
+        <is>
+          <t>Nyandoro</t>
+        </is>
+      </c>
+      <c r="D2" s="20" t="inlineStr">
+        <is>
+          <t>+17785808657</t>
+        </is>
+      </c>
+      <c r="E2" s="20" t="inlineStr">
+        <is>
+          <t>alex@michaeltenable.com</t>
+        </is>
+      </c>
+      <c r="F2" s="20" t="inlineStr">
+        <is>
+          <t>Internal Tester</t>
+        </is>
+      </c>
+      <c r="G2" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" s="21" t="n">
+        <v>5000</v>
+      </c>
+      <c r="I2" s="21" t="n">
+        <v>120000</v>
+      </c>
       <c r="J2" s="22" t="n">
         <v>120</v>
       </c>
-      <c r="K2" s="21" t="n"/>
-      <c r="L2" s="23" t="n"/>
+      <c r="K2" s="21">
+        <f>IF(J2=0,"",ROUND((I2-H2)/J2,2))</f>
+        <v/>
+      </c>
+      <c r="L2" s="23" t="n">
+        <v>46147</v>
+      </c>
       <c r="M2" s="21" t="n"/>
       <c r="N2" s="21" t="n"/>
       <c r="O2" s="21" t="n"/>
@@ -1623,15 +1658,15 @@
       <c r="EB2" s="21" t="n"/>
       <c r="EC2" s="21" t="n"/>
       <c r="ED2" s="24">
-        <f>SUM(M2:EB2)</f>
+        <f>H2+SUM(M2:EB2)</f>
         <v/>
       </c>
       <c r="EE2" s="24">
-        <f>I2-ED2</f>
+        <f>I2-H2-SUM(M2:EB2)</f>
         <v/>
       </c>
       <c r="EF2" s="25">
-        <f>IF(I2=0,"",ED2/I2)</f>
+        <f>IF(I2=0,"",(H2+SUM(M2:EB2))/I2)</f>
         <v/>
       </c>
       <c r="EG2" s="26" t="n"/>
@@ -1780,15 +1815,15 @@
       <c r="EB3" s="21" t="n"/>
       <c r="EC3" s="21" t="n"/>
       <c r="ED3" s="24">
-        <f>SUM(M3:EB3)</f>
+        <f>H3+SUM(M3:EB3)</f>
         <v/>
       </c>
       <c r="EE3" s="24">
-        <f>I3-ED3</f>
+        <f>I3-H3-SUM(M3:EB3)</f>
         <v/>
       </c>
       <c r="EF3" s="25">
-        <f>IF(I3=0,"",ED3/I3)</f>
+        <f>IF(I3=0,"",(H3+SUM(M3:EB3))/I3)</f>
         <v/>
       </c>
       <c r="EG3" s="26" t="n"/>
@@ -1937,15 +1972,15 @@
       <c r="EB4" s="21" t="n"/>
       <c r="EC4" s="21" t="n"/>
       <c r="ED4" s="24">
-        <f>SUM(M4:EB4)</f>
+        <f>H4+SUM(M4:EB4)</f>
         <v/>
       </c>
       <c r="EE4" s="24">
-        <f>I4-ED4</f>
+        <f>I4-H4-SUM(M4:EB4)</f>
         <v/>
       </c>
       <c r="EF4" s="25">
-        <f>IF(I4=0,"",ED4/I4)</f>
+        <f>IF(I4=0,"",(H4+SUM(M4:EB4))/I4)</f>
         <v/>
       </c>
       <c r="EG4" s="26" t="n"/>
@@ -2094,15 +2129,15 @@
       <c r="EB5" s="21" t="n"/>
       <c r="EC5" s="21" t="n"/>
       <c r="ED5" s="24">
-        <f>SUM(M5:EB5)</f>
+        <f>H5+SUM(M5:EB5)</f>
         <v/>
       </c>
       <c r="EE5" s="24">
-        <f>I5-ED5</f>
+        <f>I5-H5-SUM(M5:EB5)</f>
         <v/>
       </c>
       <c r="EF5" s="25">
-        <f>IF(I5=0,"",ED5/I5)</f>
+        <f>IF(I5=0,"",(H5+SUM(M5:EB5))/I5)</f>
         <v/>
       </c>
       <c r="EG5" s="26" t="n"/>
@@ -2251,15 +2286,15 @@
       <c r="EB6" s="21" t="n"/>
       <c r="EC6" s="21" t="n"/>
       <c r="ED6" s="24">
-        <f>SUM(M6:EB6)</f>
+        <f>H6+SUM(M6:EB6)</f>
         <v/>
       </c>
       <c r="EE6" s="24">
-        <f>I6-ED6</f>
+        <f>I6-H6-SUM(M6:EB6)</f>
         <v/>
       </c>
       <c r="EF6" s="25">
-        <f>IF(I6=0,"",ED6/I6)</f>
+        <f>IF(I6=0,"",(H6+SUM(M6:EB6))/I6)</f>
         <v/>
       </c>
       <c r="EG6" s="26" t="n"/>
@@ -2408,15 +2443,15 @@
       <c r="EB7" s="21" t="n"/>
       <c r="EC7" s="21" t="n"/>
       <c r="ED7" s="24">
-        <f>SUM(M7:EB7)</f>
+        <f>H7+SUM(M7:EB7)</f>
         <v/>
       </c>
       <c r="EE7" s="24">
-        <f>I7-ED7</f>
+        <f>I7-H7-SUM(M7:EB7)</f>
         <v/>
       </c>
       <c r="EF7" s="25">
-        <f>IF(I7=0,"",ED7/I7)</f>
+        <f>IF(I7=0,"",(H7+SUM(M7:EB7))/I7)</f>
         <v/>
       </c>
       <c r="EG7" s="26" t="n"/>
@@ -2565,15 +2600,15 @@
       <c r="EB8" s="21" t="n"/>
       <c r="EC8" s="21" t="n"/>
       <c r="ED8" s="24">
-        <f>SUM(M8:EB8)</f>
+        <f>H8+SUM(M8:EB8)</f>
         <v/>
       </c>
       <c r="EE8" s="24">
-        <f>I8-ED8</f>
+        <f>I8-H8-SUM(M8:EB8)</f>
         <v/>
       </c>
       <c r="EF8" s="25">
-        <f>IF(I8=0,"",ED8/I8)</f>
+        <f>IF(I8=0,"",(H8+SUM(M8:EB8))/I8)</f>
         <v/>
       </c>
       <c r="EG8" s="26" t="n"/>
@@ -2722,15 +2757,15 @@
       <c r="EB9" s="21" t="n"/>
       <c r="EC9" s="21" t="n"/>
       <c r="ED9" s="24">
-        <f>SUM(M9:EB9)</f>
+        <f>H9+SUM(M9:EB9)</f>
         <v/>
       </c>
       <c r="EE9" s="24">
-        <f>I9-ED9</f>
+        <f>I9-H9-SUM(M9:EB9)</f>
         <v/>
       </c>
       <c r="EF9" s="25">
-        <f>IF(I9=0,"",ED9/I9)</f>
+        <f>IF(I9=0,"",(H9+SUM(M9:EB9))/I9)</f>
         <v/>
       </c>
       <c r="EG9" s="26" t="n"/>
@@ -2879,15 +2914,15 @@
       <c r="EB10" s="21" t="n"/>
       <c r="EC10" s="21" t="n"/>
       <c r="ED10" s="24">
-        <f>SUM(M10:EB10)</f>
+        <f>H10+SUM(M10:EB10)</f>
         <v/>
       </c>
       <c r="EE10" s="24">
-        <f>I10-ED10</f>
+        <f>I10-H10-SUM(M10:EB10)</f>
         <v/>
       </c>
       <c r="EF10" s="25">
-        <f>IF(I10=0,"",ED10/I10)</f>
+        <f>IF(I10=0,"",(H10+SUM(M10:EB10))/I10)</f>
         <v/>
       </c>
       <c r="EG10" s="26" t="n"/>
@@ -3036,15 +3071,15 @@
       <c r="EB11" s="21" t="n"/>
       <c r="EC11" s="21" t="n"/>
       <c r="ED11" s="24">
-        <f>SUM(M11:EB11)</f>
+        <f>H11+SUM(M11:EB11)</f>
         <v/>
       </c>
       <c r="EE11" s="24">
-        <f>I11-ED11</f>
+        <f>I11-H11-SUM(M11:EB11)</f>
         <v/>
       </c>
       <c r="EF11" s="25">
-        <f>IF(I11=0,"",ED11/I11)</f>
+        <f>IF(I11=0,"",(H11+SUM(M11:EB11))/I11)</f>
         <v/>
       </c>
       <c r="EG11" s="26" t="n"/>
@@ -3193,15 +3228,15 @@
       <c r="EB12" s="21" t="n"/>
       <c r="EC12" s="21" t="n"/>
       <c r="ED12" s="24">
-        <f>SUM(M12:EB12)</f>
+        <f>H12+SUM(M12:EB12)</f>
         <v/>
       </c>
       <c r="EE12" s="24">
-        <f>I12-ED12</f>
+        <f>I12-H12-SUM(M12:EB12)</f>
         <v/>
       </c>
       <c r="EF12" s="25">
-        <f>IF(I12=0,"",ED12/I12)</f>
+        <f>IF(I12=0,"",(H12+SUM(M12:EB12))/I12)</f>
         <v/>
       </c>
       <c r="EG12" s="26" t="n"/>
@@ -3350,15 +3385,15 @@
       <c r="EB13" s="21" t="n"/>
       <c r="EC13" s="21" t="n"/>
       <c r="ED13" s="24">
-        <f>SUM(M13:EB13)</f>
+        <f>H13+SUM(M13:EB13)</f>
         <v/>
       </c>
       <c r="EE13" s="24">
-        <f>I13-ED13</f>
+        <f>I13-H13-SUM(M13:EB13)</f>
         <v/>
       </c>
       <c r="EF13" s="25">
-        <f>IF(I13=0,"",ED13/I13)</f>
+        <f>IF(I13=0,"",(H13+SUM(M13:EB13))/I13)</f>
         <v/>
       </c>
       <c r="EG13" s="26" t="n"/>
@@ -3507,15 +3542,15 @@
       <c r="EB14" s="21" t="n"/>
       <c r="EC14" s="21" t="n"/>
       <c r="ED14" s="24">
-        <f>SUM(M14:EB14)</f>
+        <f>H14+SUM(M14:EB14)</f>
         <v/>
       </c>
       <c r="EE14" s="24">
-        <f>I14-ED14</f>
+        <f>I14-H14-SUM(M14:EB14)</f>
         <v/>
       </c>
       <c r="EF14" s="25">
-        <f>IF(I14=0,"",ED14/I14)</f>
+        <f>IF(I14=0,"",(H14+SUM(M14:EB14))/I14)</f>
         <v/>
       </c>
       <c r="EG14" s="26" t="n"/>
@@ -3664,15 +3699,15 @@
       <c r="EB15" s="21" t="n"/>
       <c r="EC15" s="21" t="n"/>
       <c r="ED15" s="24">
-        <f>SUM(M15:EB15)</f>
+        <f>H15+SUM(M15:EB15)</f>
         <v/>
       </c>
       <c r="EE15" s="24">
-        <f>I15-ED15</f>
+        <f>I15-H15-SUM(M15:EB15)</f>
         <v/>
       </c>
       <c r="EF15" s="25">
-        <f>IF(I15=0,"",ED15/I15)</f>
+        <f>IF(I15=0,"",(H15+SUM(M15:EB15))/I15)</f>
         <v/>
       </c>
       <c r="EG15" s="26" t="n"/>
@@ -3821,15 +3856,15 @@
       <c r="EB16" s="21" t="n"/>
       <c r="EC16" s="21" t="n"/>
       <c r="ED16" s="24">
-        <f>SUM(M16:EB16)</f>
+        <f>H16+SUM(M16:EB16)</f>
         <v/>
       </c>
       <c r="EE16" s="24">
-        <f>I16-ED16</f>
+        <f>I16-H16-SUM(M16:EB16)</f>
         <v/>
       </c>
       <c r="EF16" s="25">
-        <f>IF(I16=0,"",ED16/I16)</f>
+        <f>IF(I16=0,"",(H16+SUM(M16:EB16))/I16)</f>
         <v/>
       </c>
       <c r="EG16" s="26" t="n"/>
@@ -3978,15 +4013,15 @@
       <c r="EB17" s="21" t="n"/>
       <c r="EC17" s="21" t="n"/>
       <c r="ED17" s="24">
-        <f>SUM(M17:EB17)</f>
+        <f>H17+SUM(M17:EB17)</f>
         <v/>
       </c>
       <c r="EE17" s="24">
-        <f>I17-ED17</f>
+        <f>I17-H17-SUM(M17:EB17)</f>
         <v/>
       </c>
       <c r="EF17" s="25">
-        <f>IF(I17=0,"",ED17/I17)</f>
+        <f>IF(I17=0,"",(H17+SUM(M17:EB17))/I17)</f>
         <v/>
       </c>
       <c r="EG17" s="26" t="n"/>
@@ -4135,15 +4170,15 @@
       <c r="EB18" s="21" t="n"/>
       <c r="EC18" s="21" t="n"/>
       <c r="ED18" s="24">
-        <f>SUM(M18:EB18)</f>
+        <f>H18+SUM(M18:EB18)</f>
         <v/>
       </c>
       <c r="EE18" s="24">
-        <f>I18-ED18</f>
+        <f>I18-H18-SUM(M18:EB18)</f>
         <v/>
       </c>
       <c r="EF18" s="25">
-        <f>IF(I18=0,"",ED18/I18)</f>
+        <f>IF(I18=0,"",(H18+SUM(M18:EB18))/I18)</f>
         <v/>
       </c>
       <c r="EG18" s="26" t="n"/>
@@ -4292,15 +4327,15 @@
       <c r="EB19" s="21" t="n"/>
       <c r="EC19" s="21" t="n"/>
       <c r="ED19" s="24">
-        <f>SUM(M19:EB19)</f>
+        <f>H19+SUM(M19:EB19)</f>
         <v/>
       </c>
       <c r="EE19" s="24">
-        <f>I19-ED19</f>
+        <f>I19-H19-SUM(M19:EB19)</f>
         <v/>
       </c>
       <c r="EF19" s="25">
-        <f>IF(I19=0,"",ED19/I19)</f>
+        <f>IF(I19=0,"",(H19+SUM(M19:EB19))/I19)</f>
         <v/>
       </c>
       <c r="EG19" s="26" t="n"/>
@@ -4449,15 +4484,15 @@
       <c r="EB20" s="21" t="n"/>
       <c r="EC20" s="21" t="n"/>
       <c r="ED20" s="24">
-        <f>SUM(M20:EB20)</f>
+        <f>H20+SUM(M20:EB20)</f>
         <v/>
       </c>
       <c r="EE20" s="24">
-        <f>I20-ED20</f>
+        <f>I20-H20-SUM(M20:EB20)</f>
         <v/>
       </c>
       <c r="EF20" s="25">
-        <f>IF(I20=0,"",ED20/I20)</f>
+        <f>IF(I20=0,"",(H20+SUM(M20:EB20))/I20)</f>
         <v/>
       </c>
       <c r="EG20" s="26" t="n"/>
@@ -4606,15 +4641,15 @@
       <c r="EB21" s="21" t="n"/>
       <c r="EC21" s="21" t="n"/>
       <c r="ED21" s="24">
-        <f>SUM(M21:EB21)</f>
+        <f>H21+SUM(M21:EB21)</f>
         <v/>
       </c>
       <c r="EE21" s="24">
-        <f>I21-ED21</f>
+        <f>I21-H21-SUM(M21:EB21)</f>
         <v/>
       </c>
       <c r="EF21" s="25">
-        <f>IF(I21=0,"",ED21/I21)</f>
+        <f>IF(I21=0,"",(H21+SUM(M21:EB21))/I21)</f>
         <v/>
       </c>
       <c r="EG21" s="26" t="n"/>
@@ -4763,15 +4798,15 @@
       <c r="EB22" s="21" t="n"/>
       <c r="EC22" s="21" t="n"/>
       <c r="ED22" s="24">
-        <f>SUM(M22:EB22)</f>
+        <f>H22+SUM(M22:EB22)</f>
         <v/>
       </c>
       <c r="EE22" s="24">
-        <f>I22-ED22</f>
+        <f>I22-H22-SUM(M22:EB22)</f>
         <v/>
       </c>
       <c r="EF22" s="25">
-        <f>IF(I22=0,"",ED22/I22)</f>
+        <f>IF(I22=0,"",(H22+SUM(M22:EB22))/I22)</f>
         <v/>
       </c>
       <c r="EG22" s="26" t="n"/>
@@ -4920,15 +4955,15 @@
       <c r="EB23" s="21" t="n"/>
       <c r="EC23" s="21" t="n"/>
       <c r="ED23" s="24">
-        <f>SUM(M23:EB23)</f>
+        <f>H23+SUM(M23:EB23)</f>
         <v/>
       </c>
       <c r="EE23" s="24">
-        <f>I23-ED23</f>
+        <f>I23-H23-SUM(M23:EB23)</f>
         <v/>
       </c>
       <c r="EF23" s="25">
-        <f>IF(I23=0,"",ED23/I23)</f>
+        <f>IF(I23=0,"",(H23+SUM(M23:EB23))/I23)</f>
         <v/>
       </c>
       <c r="EG23" s="26" t="n"/>
@@ -5077,15 +5112,15 @@
       <c r="EB24" s="21" t="n"/>
       <c r="EC24" s="21" t="n"/>
       <c r="ED24" s="24">
-        <f>SUM(M24:EB24)</f>
+        <f>H24+SUM(M24:EB24)</f>
         <v/>
       </c>
       <c r="EE24" s="24">
-        <f>I24-ED24</f>
+        <f>I24-H24-SUM(M24:EB24)</f>
         <v/>
       </c>
       <c r="EF24" s="25">
-        <f>IF(I24=0,"",ED24/I24)</f>
+        <f>IF(I24=0,"",(H24+SUM(M24:EB24))/I24)</f>
         <v/>
       </c>
       <c r="EG24" s="26" t="n"/>
@@ -5234,15 +5269,15 @@
       <c r="EB25" s="21" t="n"/>
       <c r="EC25" s="21" t="n"/>
       <c r="ED25" s="24">
-        <f>SUM(M25:EB25)</f>
+        <f>H25+SUM(M25:EB25)</f>
         <v/>
       </c>
       <c r="EE25" s="24">
-        <f>I25-ED25</f>
+        <f>I25-H25-SUM(M25:EB25)</f>
         <v/>
       </c>
       <c r="EF25" s="25">
-        <f>IF(I25=0,"",ED25/I25)</f>
+        <f>IF(I25=0,"",(H25+SUM(M25:EB25))/I25)</f>
         <v/>
       </c>
       <c r="EG25" s="26" t="n"/>
@@ -5391,15 +5426,15 @@
       <c r="EB26" s="21" t="n"/>
       <c r="EC26" s="21" t="n"/>
       <c r="ED26" s="24">
-        <f>SUM(M26:EB26)</f>
+        <f>H26+SUM(M26:EB26)</f>
         <v/>
       </c>
       <c r="EE26" s="24">
-        <f>I26-ED26</f>
+        <f>I26-H26-SUM(M26:EB26)</f>
         <v/>
       </c>
       <c r="EF26" s="25">
-        <f>IF(I26=0,"",ED26/I26)</f>
+        <f>IF(I26=0,"",(H26+SUM(M26:EB26))/I26)</f>
         <v/>
       </c>
       <c r="EG26" s="26" t="n"/>
@@ -5548,15 +5583,15 @@
       <c r="EB27" s="21" t="n"/>
       <c r="EC27" s="21" t="n"/>
       <c r="ED27" s="24">
-        <f>SUM(M27:EB27)</f>
+        <f>H27+SUM(M27:EB27)</f>
         <v/>
       </c>
       <c r="EE27" s="24">
-        <f>I27-ED27</f>
+        <f>I27-H27-SUM(M27:EB27)</f>
         <v/>
       </c>
       <c r="EF27" s="25">
-        <f>IF(I27=0,"",ED27/I27)</f>
+        <f>IF(I27=0,"",(H27+SUM(M27:EB27))/I27)</f>
         <v/>
       </c>
       <c r="EG27" s="26" t="n"/>
@@ -5705,15 +5740,15 @@
       <c r="EB28" s="21" t="n"/>
       <c r="EC28" s="21" t="n"/>
       <c r="ED28" s="24">
-        <f>SUM(M28:EB28)</f>
+        <f>H28+SUM(M28:EB28)</f>
         <v/>
       </c>
       <c r="EE28" s="24">
-        <f>I28-ED28</f>
+        <f>I28-H28-SUM(M28:EB28)</f>
         <v/>
       </c>
       <c r="EF28" s="25">
-        <f>IF(I28=0,"",ED28/I28)</f>
+        <f>IF(I28=0,"",(H28+SUM(M28:EB28))/I28)</f>
         <v/>
       </c>
       <c r="EG28" s="26" t="n"/>
@@ -5862,15 +5897,15 @@
       <c r="EB29" s="21" t="n"/>
       <c r="EC29" s="21" t="n"/>
       <c r="ED29" s="24">
-        <f>SUM(M29:EB29)</f>
+        <f>H29+SUM(M29:EB29)</f>
         <v/>
       </c>
       <c r="EE29" s="24">
-        <f>I29-ED29</f>
+        <f>I29-H29-SUM(M29:EB29)</f>
         <v/>
       </c>
       <c r="EF29" s="25">
-        <f>IF(I29=0,"",ED29/I29)</f>
+        <f>IF(I29=0,"",(H29+SUM(M29:EB29))/I29)</f>
         <v/>
       </c>
       <c r="EG29" s="26" t="n"/>
@@ -6019,15 +6054,15 @@
       <c r="EB30" s="21" t="n"/>
       <c r="EC30" s="21" t="n"/>
       <c r="ED30" s="24">
-        <f>SUM(M30:EB30)</f>
+        <f>H30+SUM(M30:EB30)</f>
         <v/>
       </c>
       <c r="EE30" s="24">
-        <f>I30-ED30</f>
+        <f>I30-H30-SUM(M30:EB30)</f>
         <v/>
       </c>
       <c r="EF30" s="25">
-        <f>IF(I30=0,"",ED30/I30)</f>
+        <f>IF(I30=0,"",(H30+SUM(M30:EB30))/I30)</f>
         <v/>
       </c>
       <c r="EG30" s="26" t="n"/>
@@ -6176,15 +6211,15 @@
       <c r="EB31" s="21" t="n"/>
       <c r="EC31" s="21" t="n"/>
       <c r="ED31" s="24">
-        <f>SUM(M31:EB31)</f>
+        <f>H31+SUM(M31:EB31)</f>
         <v/>
       </c>
       <c r="EE31" s="24">
-        <f>I31-ED31</f>
+        <f>I31-H31-SUM(M31:EB31)</f>
         <v/>
       </c>
       <c r="EF31" s="25">
-        <f>IF(I31=0,"",ED31/I31)</f>
+        <f>IF(I31=0,"",(H31+SUM(M31:EB31))/I31)</f>
         <v/>
       </c>
       <c r="EG31" s="26" t="n"/>
@@ -6333,15 +6368,15 @@
       <c r="EB32" s="21" t="n"/>
       <c r="EC32" s="21" t="n"/>
       <c r="ED32" s="24">
-        <f>SUM(M32:EB32)</f>
+        <f>H32+SUM(M32:EB32)</f>
         <v/>
       </c>
       <c r="EE32" s="24">
-        <f>I32-ED32</f>
+        <f>I32-H32-SUM(M32:EB32)</f>
         <v/>
       </c>
       <c r="EF32" s="25">
-        <f>IF(I32=0,"",ED32/I32)</f>
+        <f>IF(I32=0,"",(H32+SUM(M32:EB32))/I32)</f>
         <v/>
       </c>
       <c r="EG32" s="26" t="n"/>
@@ -6490,15 +6525,15 @@
       <c r="EB33" s="21" t="n"/>
       <c r="EC33" s="21" t="n"/>
       <c r="ED33" s="24">
-        <f>SUM(M33:EB33)</f>
+        <f>H33+SUM(M33:EB33)</f>
         <v/>
       </c>
       <c r="EE33" s="24">
-        <f>I33-ED33</f>
+        <f>I33-H33-SUM(M33:EB33)</f>
         <v/>
       </c>
       <c r="EF33" s="25">
-        <f>IF(I33=0,"",ED33/I33)</f>
+        <f>IF(I33=0,"",(H33+SUM(M33:EB33))/I33)</f>
         <v/>
       </c>
       <c r="EG33" s="26" t="n"/>
@@ -6647,15 +6682,15 @@
       <c r="EB34" s="21" t="n"/>
       <c r="EC34" s="21" t="n"/>
       <c r="ED34" s="24">
-        <f>SUM(M34:EB34)</f>
+        <f>H34+SUM(M34:EB34)</f>
         <v/>
       </c>
       <c r="EE34" s="24">
-        <f>I34-ED34</f>
+        <f>I34-H34-SUM(M34:EB34)</f>
         <v/>
       </c>
       <c r="EF34" s="25">
-        <f>IF(I34=0,"",ED34/I34)</f>
+        <f>IF(I34=0,"",(H34+SUM(M34:EB34))/I34)</f>
         <v/>
       </c>
       <c r="EG34" s="26" t="n"/>
@@ -6804,15 +6839,15 @@
       <c r="EB35" s="21" t="n"/>
       <c r="EC35" s="21" t="n"/>
       <c r="ED35" s="24">
-        <f>SUM(M35:EB35)</f>
+        <f>H35+SUM(M35:EB35)</f>
         <v/>
       </c>
       <c r="EE35" s="24">
-        <f>I35-ED35</f>
+        <f>I35-H35-SUM(M35:EB35)</f>
         <v/>
       </c>
       <c r="EF35" s="25">
-        <f>IF(I35=0,"",ED35/I35)</f>
+        <f>IF(I35=0,"",(H35+SUM(M35:EB35))/I35)</f>
         <v/>
       </c>
       <c r="EG35" s="26" t="n"/>
@@ -6961,15 +6996,15 @@
       <c r="EB36" s="21" t="n"/>
       <c r="EC36" s="21" t="n"/>
       <c r="ED36" s="24">
-        <f>SUM(M36:EB36)</f>
+        <f>H36+SUM(M36:EB36)</f>
         <v/>
       </c>
       <c r="EE36" s="24">
-        <f>I36-ED36</f>
+        <f>I36-H36-SUM(M36:EB36)</f>
         <v/>
       </c>
       <c r="EF36" s="25">
-        <f>IF(I36=0,"",ED36/I36)</f>
+        <f>IF(I36=0,"",(H36+SUM(M36:EB36))/I36)</f>
         <v/>
       </c>
       <c r="EG36" s="26" t="n"/>
@@ -7118,15 +7153,15 @@
       <c r="EB37" s="21" t="n"/>
       <c r="EC37" s="21" t="n"/>
       <c r="ED37" s="24">
-        <f>SUM(M37:EB37)</f>
+        <f>H37+SUM(M37:EB37)</f>
         <v/>
       </c>
       <c r="EE37" s="24">
-        <f>I37-ED37</f>
+        <f>I37-H37-SUM(M37:EB37)</f>
         <v/>
       </c>
       <c r="EF37" s="25">
-        <f>IF(I37=0,"",ED37/I37)</f>
+        <f>IF(I37=0,"",(H37+SUM(M37:EB37))/I37)</f>
         <v/>
       </c>
       <c r="EG37" s="26" t="n"/>
@@ -7275,15 +7310,15 @@
       <c r="EB38" s="21" t="n"/>
       <c r="EC38" s="21" t="n"/>
       <c r="ED38" s="24">
-        <f>SUM(M38:EB38)</f>
+        <f>H38+SUM(M38:EB38)</f>
         <v/>
       </c>
       <c r="EE38" s="24">
-        <f>I38-ED38</f>
+        <f>I38-H38-SUM(M38:EB38)</f>
         <v/>
       </c>
       <c r="EF38" s="25">
-        <f>IF(I38=0,"",ED38/I38)</f>
+        <f>IF(I38=0,"",(H38+SUM(M38:EB38))/I38)</f>
         <v/>
       </c>
       <c r="EG38" s="26" t="n"/>
@@ -7432,15 +7467,15 @@
       <c r="EB39" s="21" t="n"/>
       <c r="EC39" s="21" t="n"/>
       <c r="ED39" s="24">
-        <f>SUM(M39:EB39)</f>
+        <f>H39+SUM(M39:EB39)</f>
         <v/>
       </c>
       <c r="EE39" s="24">
-        <f>I39-ED39</f>
+        <f>I39-H39-SUM(M39:EB39)</f>
         <v/>
       </c>
       <c r="EF39" s="25">
-        <f>IF(I39=0,"",ED39/I39)</f>
+        <f>IF(I39=0,"",(H39+SUM(M39:EB39))/I39)</f>
         <v/>
       </c>
       <c r="EG39" s="26" t="n"/>
@@ -7589,15 +7624,15 @@
       <c r="EB40" s="21" t="n"/>
       <c r="EC40" s="21" t="n"/>
       <c r="ED40" s="24">
-        <f>SUM(M40:EB40)</f>
+        <f>H40+SUM(M40:EB40)</f>
         <v/>
       </c>
       <c r="EE40" s="24">
-        <f>I40-ED40</f>
+        <f>I40-H40-SUM(M40:EB40)</f>
         <v/>
       </c>
       <c r="EF40" s="25">
-        <f>IF(I40=0,"",ED40/I40)</f>
+        <f>IF(I40=0,"",(H40+SUM(M40:EB40))/I40)</f>
         <v/>
       </c>
       <c r="EG40" s="26" t="n"/>
@@ -7746,15 +7781,15 @@
       <c r="EB41" s="21" t="n"/>
       <c r="EC41" s="21" t="n"/>
       <c r="ED41" s="24">
-        <f>SUM(M41:EB41)</f>
+        <f>H41+SUM(M41:EB41)</f>
         <v/>
       </c>
       <c r="EE41" s="24">
-        <f>I41-ED41</f>
+        <f>I41-H41-SUM(M41:EB41)</f>
         <v/>
       </c>
       <c r="EF41" s="25">
-        <f>IF(I41=0,"",ED41/I41)</f>
+        <f>IF(I41=0,"",(H41+SUM(M41:EB41))/I41)</f>
         <v/>
       </c>
       <c r="EG41" s="26" t="n"/>
@@ -7903,15 +7938,15 @@
       <c r="EB42" s="21" t="n"/>
       <c r="EC42" s="21" t="n"/>
       <c r="ED42" s="24">
-        <f>SUM(M42:EB42)</f>
+        <f>H42+SUM(M42:EB42)</f>
         <v/>
       </c>
       <c r="EE42" s="24">
-        <f>I42-ED42</f>
+        <f>I42-H42-SUM(M42:EB42)</f>
         <v/>
       </c>
       <c r="EF42" s="25">
-        <f>IF(I42=0,"",ED42/I42)</f>
+        <f>IF(I42=0,"",(H42+SUM(M42:EB42))/I42)</f>
         <v/>
       </c>
       <c r="EG42" s="26" t="n"/>
@@ -8060,15 +8095,15 @@
       <c r="EB43" s="21" t="n"/>
       <c r="EC43" s="21" t="n"/>
       <c r="ED43" s="24">
-        <f>SUM(M43:EB43)</f>
+        <f>H43+SUM(M43:EB43)</f>
         <v/>
       </c>
       <c r="EE43" s="24">
-        <f>I43-ED43</f>
+        <f>I43-H43-SUM(M43:EB43)</f>
         <v/>
       </c>
       <c r="EF43" s="25">
-        <f>IF(I43=0,"",ED43/I43)</f>
+        <f>IF(I43=0,"",(H43+SUM(M43:EB43))/I43)</f>
         <v/>
       </c>
       <c r="EG43" s="26" t="n"/>
@@ -8217,15 +8252,15 @@
       <c r="EB44" s="21" t="n"/>
       <c r="EC44" s="21" t="n"/>
       <c r="ED44" s="24">
-        <f>SUM(M44:EB44)</f>
+        <f>H44+SUM(M44:EB44)</f>
         <v/>
       </c>
       <c r="EE44" s="24">
-        <f>I44-ED44</f>
+        <f>I44-H44-SUM(M44:EB44)</f>
         <v/>
       </c>
       <c r="EF44" s="25">
-        <f>IF(I44=0,"",ED44/I44)</f>
+        <f>IF(I44=0,"",(H44+SUM(M44:EB44))/I44)</f>
         <v/>
       </c>
       <c r="EG44" s="26" t="n"/>
@@ -8374,15 +8409,15 @@
       <c r="EB45" s="21" t="n"/>
       <c r="EC45" s="21" t="n"/>
       <c r="ED45" s="24">
-        <f>SUM(M45:EB45)</f>
+        <f>H45+SUM(M45:EB45)</f>
         <v/>
       </c>
       <c r="EE45" s="24">
-        <f>I45-ED45</f>
+        <f>I45-H45-SUM(M45:EB45)</f>
         <v/>
       </c>
       <c r="EF45" s="25">
-        <f>IF(I45=0,"",ED45/I45)</f>
+        <f>IF(I45=0,"",(H45+SUM(M45:EB45))/I45)</f>
         <v/>
       </c>
       <c r="EG45" s="26" t="n"/>
@@ -8531,15 +8566,15 @@
       <c r="EB46" s="21" t="n"/>
       <c r="EC46" s="21" t="n"/>
       <c r="ED46" s="24">
-        <f>SUM(M46:EB46)</f>
+        <f>H46+SUM(M46:EB46)</f>
         <v/>
       </c>
       <c r="EE46" s="24">
-        <f>I46-ED46</f>
+        <f>I46-H46-SUM(M46:EB46)</f>
         <v/>
       </c>
       <c r="EF46" s="25">
-        <f>IF(I46=0,"",ED46/I46)</f>
+        <f>IF(I46=0,"",(H46+SUM(M46:EB46))/I46)</f>
         <v/>
       </c>
       <c r="EG46" s="26" t="n"/>
@@ -8688,15 +8723,15 @@
       <c r="EB47" s="21" t="n"/>
       <c r="EC47" s="21" t="n"/>
       <c r="ED47" s="24">
-        <f>SUM(M47:EB47)</f>
+        <f>H47+SUM(M47:EB47)</f>
         <v/>
       </c>
       <c r="EE47" s="24">
-        <f>I47-ED47</f>
+        <f>I47-H47-SUM(M47:EB47)</f>
         <v/>
       </c>
       <c r="EF47" s="25">
-        <f>IF(I47=0,"",ED47/I47)</f>
+        <f>IF(I47=0,"",(H47+SUM(M47:EB47))/I47)</f>
         <v/>
       </c>
       <c r="EG47" s="26" t="n"/>
@@ -8845,15 +8880,15 @@
       <c r="EB48" s="21" t="n"/>
       <c r="EC48" s="21" t="n"/>
       <c r="ED48" s="24">
-        <f>SUM(M48:EB48)</f>
+        <f>H48+SUM(M48:EB48)</f>
         <v/>
       </c>
       <c r="EE48" s="24">
-        <f>I48-ED48</f>
+        <f>I48-H48-SUM(M48:EB48)</f>
         <v/>
       </c>
       <c r="EF48" s="25">
-        <f>IF(I48=0,"",ED48/I48)</f>
+        <f>IF(I48=0,"",(H48+SUM(M48:EB48))/I48)</f>
         <v/>
       </c>
       <c r="EG48" s="26" t="n"/>
@@ -9002,15 +9037,15 @@
       <c r="EB49" s="21" t="n"/>
       <c r="EC49" s="21" t="n"/>
       <c r="ED49" s="24">
-        <f>SUM(M49:EB49)</f>
+        <f>H49+SUM(M49:EB49)</f>
         <v/>
       </c>
       <c r="EE49" s="24">
-        <f>I49-ED49</f>
+        <f>I49-H49-SUM(M49:EB49)</f>
         <v/>
       </c>
       <c r="EF49" s="25">
-        <f>IF(I49=0,"",ED49/I49)</f>
+        <f>IF(I49=0,"",(H49+SUM(M49:EB49))/I49)</f>
         <v/>
       </c>
       <c r="EG49" s="26" t="n"/>
@@ -9159,15 +9194,15 @@
       <c r="EB50" s="21" t="n"/>
       <c r="EC50" s="21" t="n"/>
       <c r="ED50" s="24">
-        <f>SUM(M50:EB50)</f>
+        <f>H50+SUM(M50:EB50)</f>
         <v/>
       </c>
       <c r="EE50" s="24">
-        <f>I50-ED50</f>
+        <f>I50-H50-SUM(M50:EB50)</f>
         <v/>
       </c>
       <c r="EF50" s="25">
-        <f>IF(I50=0,"",ED50/I50)</f>
+        <f>IF(I50=0,"",(H50+SUM(M50:EB50))/I50)</f>
         <v/>
       </c>
       <c r="EG50" s="26" t="n"/>
@@ -9316,15 +9351,15 @@
       <c r="EB51" s="21" t="n"/>
       <c r="EC51" s="21" t="n"/>
       <c r="ED51" s="24">
-        <f>SUM(M51:EB51)</f>
+        <f>H51+SUM(M51:EB51)</f>
         <v/>
       </c>
       <c r="EE51" s="24">
-        <f>I51-ED51</f>
+        <f>I51-H51-SUM(M51:EB51)</f>
         <v/>
       </c>
       <c r="EF51" s="25">
-        <f>IF(I51=0,"",ED51/I51)</f>
+        <f>IF(I51=0,"",(H51+SUM(M51:EB51))/I51)</f>
         <v/>
       </c>
       <c r="EG51" s="26" t="n"/>

</xml_diff>